<commit_message>
Cleaning up preprocessing file
</commit_message>
<xml_diff>
--- a/data/French_Post_Survey.xlsx
+++ b/data/French_Post_Survey.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\ST558\ST542_Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\ST558\ST542_Project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C910874F-4BF8-49AA-A406-1D4C980281F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7051BA-694E-47E6-973B-0F3EFC8E6592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4147" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4139" uniqueCount="421">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1368,25 +1368,13 @@
     <t>cpspruil@ncsu.edu</t>
   </si>
   <si>
-    <t>wdepue@ncsu.edu</t>
-  </si>
-  <si>
     <t>klburns3@ncsu.edu</t>
   </si>
   <si>
     <t>sryan3@ncsu.edu</t>
   </si>
   <si>
-    <t>French, Arts and architecture, Art entrepreneurship</t>
-  </si>
-  <si>
     <t>knjoyner@ncsu.edu</t>
-  </si>
-  <si>
-    <t>Social Science</t>
-  </si>
-  <si>
-    <t>hkarring@ncsu.edu</t>
   </si>
   <si>
     <t>Social Science, Language other than French</t>
@@ -1421,18 +1409,12 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFF2CC"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1447,7 +1429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1456,7 +1438,8 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1675,7 +1658,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:CC71"/>
+  <dimension ref="A1:CF73"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="84" width="18.85546875" customWidth="1"/>
@@ -9156,7 +9139,7 @@
         <v>361727604</v>
       </c>
     </row>
-    <row r="33" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>45483.863208622686</v>
       </c>
@@ -9389,7 +9372,7 @@
         <v>113827207</v>
       </c>
     </row>
-    <row r="34" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>45484.432426331019</v>
       </c>
@@ -9619,7 +9602,7 @@
         <v>433627616</v>
       </c>
     </row>
-    <row r="35" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>45484.74011337963</v>
       </c>
@@ -9852,7 +9835,7 @@
         <v>81727693</v>
       </c>
     </row>
-    <row r="36" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>45488.590129953707</v>
       </c>
@@ -10085,7 +10068,7 @@
         <v>672828210</v>
       </c>
     </row>
-    <row r="37" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>45493.464063159721</v>
       </c>
@@ -10314,8 +10297,9 @@
       <c r="BZ37" s="1">
         <v>3007272782</v>
       </c>
+      <c r="CC37" s="7"/>
     </row>
-    <row r="38" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>45583.748659178236</v>
       </c>
@@ -10544,8 +10528,9 @@
       <c r="BZ38" s="1">
         <v>51327502</v>
       </c>
+      <c r="CC38" s="7"/>
     </row>
-    <row r="39" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>45583.839191747684</v>
       </c>
@@ -10777,8 +10762,9 @@
       <c r="BZ39" s="1" t="s">
         <v>324</v>
       </c>
+      <c r="CC39" s="7"/>
     </row>
-    <row r="40" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>45584.586853298606</v>
       </c>
@@ -11007,8 +10993,10 @@
       <c r="BZ40" s="1">
         <v>302627607</v>
       </c>
+      <c r="CC40" s="7"/>
+      <c r="CF40" s="7"/>
     </row>
-    <row r="41" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>45585.562540023151</v>
       </c>
@@ -11237,8 +11225,10 @@
       <c r="BZ41" s="1">
         <v>672828210</v>
       </c>
+      <c r="CC41" s="7"/>
+      <c r="CF41" s="7"/>
     </row>
-    <row r="42" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>45587.685891099536</v>
       </c>
@@ -11470,8 +11460,10 @@
       <c r="BZ42" s="1">
         <v>772427332</v>
       </c>
+      <c r="CC42" s="7"/>
+      <c r="CF42" s="7"/>
     </row>
-    <row r="43" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>45843.614259965281</v>
       </c>
@@ -11712,8 +11704,9 @@
       <c r="CC43" s="6" t="s">
         <v>343</v>
       </c>
+      <c r="CF43" s="7"/>
     </row>
-    <row r="44" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>45843.65740394676</v>
       </c>
@@ -11944,9 +11937,10 @@
       </c>
       <c r="CA44" s="4"/>
       <c r="CB44" s="5"/>
-      <c r="CC44" s="5"/>
+      <c r="CC44" s="6"/>
+      <c r="CF44" s="7"/>
     </row>
-    <row r="45" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>45844.406656342588</v>
       </c>
@@ -12179,16 +12173,17 @@
         <v>280528403</v>
       </c>
       <c r="CA45" s="4">
-        <v>153027023</v>
+        <v>280528403</v>
       </c>
       <c r="CB45" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="CC45" s="5" t="s">
-        <v>351</v>
-      </c>
+        <v>372</v>
+      </c>
+      <c r="CC45" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="CF45" s="7"/>
     </row>
-    <row r="46" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>45844.528457986111</v>
       </c>
@@ -12421,16 +12416,19 @@
         <v>13227529</v>
       </c>
       <c r="CA46" s="4">
-        <v>331427858</v>
+        <v>13227529</v>
       </c>
       <c r="CB46" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="CC46" s="5" t="s">
-        <v>358</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="CC46" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="CD46" s="4"/>
+      <c r="CE46" s="5"/>
+      <c r="CF46" s="6"/>
     </row>
-    <row r="47" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>45846.657795462961</v>
       </c>
@@ -12671,8 +12669,11 @@
       <c r="CC47" s="6" t="s">
         <v>363</v>
       </c>
+      <c r="CD47" s="4"/>
+      <c r="CE47" s="5"/>
+      <c r="CF47" s="6"/>
     </row>
-    <row r="48" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>45848.318449421291</v>
       </c>
@@ -12905,16 +12906,17 @@
         <v>1311427292</v>
       </c>
       <c r="CA48" s="4">
-        <v>651427410</v>
+        <v>1311427292</v>
       </c>
       <c r="CB48" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="CC48" s="5" t="s">
-        <v>369</v>
-      </c>
+      <c r="CC48" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="CF48" s="7"/>
     </row>
-    <row r="49" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>45849.315706400463</v>
       </c>
@@ -13144,16 +13146,17 @@
         <v>651427410</v>
       </c>
       <c r="CA49" s="4">
-        <v>280528403</v>
+        <v>651427410</v>
       </c>
       <c r="CB49" s="5" t="s">
-        <v>372</v>
+        <v>102</v>
       </c>
       <c r="CC49" s="6" t="s">
-        <v>373</v>
-      </c>
+        <v>369</v>
+      </c>
+      <c r="CF49" s="7"/>
     </row>
-    <row r="50" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>45850.714447974533</v>
       </c>
@@ -13385,17 +13388,14 @@
       <c r="BZ50" s="1">
         <v>51627513</v>
       </c>
-      <c r="CA50" s="4">
-        <v>280528403</v>
-      </c>
-      <c r="CB50" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="CC50" s="5" t="s">
-        <v>373</v>
-      </c>
+      <c r="CA50" s="4"/>
+      <c r="CB50" s="5"/>
+      <c r="CC50" s="6"/>
+      <c r="CD50" s="4"/>
+      <c r="CE50" s="5"/>
+      <c r="CF50" s="6"/>
     </row>
-    <row r="51" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>45852.866202002318</v>
       </c>
@@ -13625,16 +13625,17 @@
         <v>90427713</v>
       </c>
       <c r="CA51" s="4">
-        <v>300027519</v>
+        <v>90427713</v>
       </c>
       <c r="CB51" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="CC51" s="5" t="s">
-        <v>380</v>
-      </c>
+        <v>419</v>
+      </c>
+      <c r="CC51" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="CF51" s="7"/>
     </row>
-    <row r="52" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>45860.617359027776</v>
       </c>
@@ -13863,8 +13864,18 @@
       <c r="BZ52" s="1">
         <v>3009</v>
       </c>
+      <c r="CA52" s="4">
+        <v>300927607</v>
+      </c>
+      <c r="CB52" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="CC52" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="CF52" s="7"/>
     </row>
-    <row r="53" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>45860.623097233794</v>
       </c>
@@ -14093,8 +14104,18 @@
       <c r="BZ53" s="1">
         <v>153027023</v>
       </c>
+      <c r="CA53" s="4">
+        <v>153027023</v>
+      </c>
+      <c r="CB53" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="CC53" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="CF53" s="7"/>
     </row>
-    <row r="54" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
         <v>45860.624873668981</v>
       </c>
@@ -14323,8 +14344,18 @@
       <c r="BZ54" s="1">
         <v>300027519</v>
       </c>
+      <c r="CA54" s="4">
+        <v>300027519</v>
+      </c>
+      <c r="CB54" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="CC54" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="CF54" s="7"/>
     </row>
-    <row r="55" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
         <v>45860.642098321754</v>
       </c>
@@ -14553,8 +14584,18 @@
       <c r="BZ55" s="1">
         <v>331427858</v>
       </c>
+      <c r="CA55" s="4">
+        <v>331427858</v>
+      </c>
+      <c r="CB55" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="CC55" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="CF55" s="7"/>
     </row>
-    <row r="56" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
         <v>45860.64557231481</v>
       </c>
@@ -14786,8 +14827,9 @@
       <c r="BZ56" s="1">
         <v>27607</v>
       </c>
+      <c r="CC56" s="7"/>
     </row>
-    <row r="57" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>45860.650165011575</v>
       </c>
@@ -15019,8 +15061,17 @@
       <c r="BZ57" s="1">
         <v>210527603</v>
       </c>
+      <c r="CA57" s="4">
+        <v>210537603</v>
+      </c>
+      <c r="CB57" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="CC57" s="6" t="s">
+        <v>418</v>
+      </c>
     </row>
-    <row r="58" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>45860.667371736112</v>
       </c>
@@ -15252,8 +15303,9 @@
       <c r="BZ58" s="1">
         <v>42328658</v>
       </c>
+      <c r="CC58" s="7"/>
     </row>
-    <row r="59" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
         <v>45860.74661318287</v>
       </c>
@@ -15485,8 +15537,17 @@
       <c r="BZ59" s="1">
         <v>210627886</v>
       </c>
+      <c r="CA59" s="4">
+        <v>210627886</v>
+      </c>
+      <c r="CB59" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="CC59" s="6" t="s">
+        <v>415</v>
+      </c>
     </row>
-    <row r="60" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
         <v>45860.848506736111</v>
       </c>
@@ -15715,8 +15776,9 @@
       <c r="BZ60" s="1">
         <v>27609</v>
       </c>
+      <c r="CC60" s="7"/>
     </row>
-    <row r="61" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>45861.829185451388</v>
       </c>
@@ -15945,8 +16007,9 @@
       <c r="BZ61" s="1">
         <v>113027603</v>
       </c>
+      <c r="CC61" s="7"/>
     </row>
-    <row r="62" spans="1:81" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
         <v>45861.970749386572</v>
       </c>
@@ -16175,105 +16238,58 @@
       <c r="BZ62" s="1">
         <v>24927979</v>
       </c>
+      <c r="CC62" s="7"/>
     </row>
-    <row r="63" spans="1:81" x14ac:dyDescent="0.2">
-      <c r="CA63" s="4">
-        <v>300927607</v>
-      </c>
-      <c r="CB63" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="CC63" s="5" t="s">
-        <v>414</v>
-      </c>
+    <row r="63" spans="1:84" x14ac:dyDescent="0.2">
+      <c r="CA63" s="4"/>
+      <c r="CB63" s="5"/>
+      <c r="CC63" s="6"/>
     </row>
-    <row r="64" spans="1:81" x14ac:dyDescent="0.2">
-      <c r="CA64" s="4">
-        <v>210627886</v>
-      </c>
-      <c r="CB64" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="CC64" s="5" t="s">
-        <v>415</v>
-      </c>
+    <row r="64" spans="1:84" x14ac:dyDescent="0.2">
+      <c r="CA64" s="4"/>
+      <c r="CB64" s="5"/>
+      <c r="CC64" s="6"/>
     </row>
     <row r="65" spans="79:81" x14ac:dyDescent="0.2">
-      <c r="CA65" s="4">
-        <v>5327516</v>
-      </c>
-      <c r="CB65" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="CC65" s="6" t="s">
-        <v>416</v>
-      </c>
+      <c r="CA65" s="4"/>
+      <c r="CB65" s="5"/>
+      <c r="CC65" s="6"/>
     </row>
     <row r="66" spans="79:81" x14ac:dyDescent="0.2">
-      <c r="CA66" s="4">
-        <v>1311427292</v>
-      </c>
-      <c r="CB66" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="CC66" s="6" t="s">
-        <v>417</v>
-      </c>
+      <c r="CA66" s="4"/>
+      <c r="CB66" s="5"/>
+      <c r="CC66" s="6"/>
     </row>
     <row r="67" spans="79:81" x14ac:dyDescent="0.2">
-      <c r="CA67" s="4">
-        <v>13227529</v>
-      </c>
-      <c r="CB67" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="CC67" s="6" t="s">
-        <v>418</v>
-      </c>
+      <c r="CA67" s="4"/>
+      <c r="CB67" s="5"/>
+      <c r="CC67" s="6"/>
     </row>
     <row r="68" spans="79:81" x14ac:dyDescent="0.2">
-      <c r="CA68" s="4">
-        <v>140127606</v>
-      </c>
-      <c r="CB68" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="CC68" s="5" t="s">
-        <v>343</v>
-      </c>
+      <c r="CA68" s="4"/>
+      <c r="CB68" s="5"/>
+      <c r="CC68" s="6"/>
     </row>
     <row r="69" spans="79:81" x14ac:dyDescent="0.2">
-      <c r="CA69" s="4">
-        <v>210537603</v>
-      </c>
-      <c r="CB69" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="CC69" s="5" t="s">
-        <v>420</v>
-      </c>
+      <c r="CA69" s="4"/>
+      <c r="CB69" s="5"/>
+      <c r="CC69" s="6"/>
     </row>
     <row r="70" spans="79:81" x14ac:dyDescent="0.2">
-      <c r="CA70" s="4">
-        <v>49529414</v>
-      </c>
-      <c r="CB70" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="CC70" s="5" t="s">
-        <v>422</v>
-      </c>
+      <c r="CA70" s="4"/>
+      <c r="CB70" s="5"/>
+      <c r="CC70" s="6"/>
     </row>
     <row r="71" spans="79:81" x14ac:dyDescent="0.2">
-      <c r="CA71" s="4">
-        <v>90427713</v>
-      </c>
-      <c r="CB71" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="CC71" s="6" t="s">
-        <v>424</v>
-      </c>
+      <c r="CA71" s="4"/>
+      <c r="CB71" s="5"/>
+      <c r="CC71" s="6"/>
+    </row>
+    <row r="72" spans="79:81" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="CC72" s="7"/>
+    </row>
+    <row r="73" spans="79:81" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="CC73" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>